<commit_message>
finished: Linopy workshop exercises
</commit_message>
<xml_diff>
--- a/lectures/Simplified merit order example.xlsx
+++ b/lectures/Simplified merit order example.xlsx
@@ -8,24 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://imfformacion-my.sharepoint.com/personal/fcorniellec799_alumnos_imf_com/Documents/Documentos/Desktop/17 - Projects/24 - data-science-for-esm/lectures/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="910" documentId="8_{B10321C2-96A1-42F6-B7DB-C285CE0230F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20DE2D46-8435-441B-82DF-6C5B5315D359}"/>
+  <xr:revisionPtr revIDLastSave="911" documentId="8_{B10321C2-96A1-42F6-B7DB-C285CE0230F2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{16A8232D-B888-46BB-B30D-2B81C8496BD7}"/>
   <bookViews>
-    <workbookView xWindow="-2093" yWindow="-16200" windowWidth="14565" windowHeight="15562" activeTab="1" xr2:uid="{0D21AE2B-3958-40C4-9665-512AF48DED00}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{0D21AE2B-3958-40C4-9665-512AF48DED00}"/>
   </bookViews>
   <sheets>
     <sheet name="simplified merit order" sheetId="1" r:id="rId1"/>
     <sheet name="Optimisation problem example" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlchart.v1.0" hidden="1">'Optimisation problem example'!$A$32:$A$38</definedName>
-    <definedName name="_xlchart.v1.1" hidden="1">'Optimisation problem example'!$B$31</definedName>
-    <definedName name="_xlchart.v1.2" hidden="1">'Optimisation problem example'!$B$32:$B$38</definedName>
-    <definedName name="_xlchart.v1.3" hidden="1">'Optimisation problem example'!$C$30</definedName>
-    <definedName name="_xlchart.v1.4" hidden="1">'Optimisation problem example'!$C$32:$C$33</definedName>
-    <definedName name="_xlchart.v1.5" hidden="1">'Optimisation problem example'!$D$32:$D$33</definedName>
-    <definedName name="_xlchart.v1.6" hidden="1">'Optimisation problem example'!$E$30</definedName>
-    <definedName name="_xlchart.v1.7" hidden="1">'Optimisation problem example'!$E$32</definedName>
-    <definedName name="_xlchart.v1.8" hidden="1">'Optimisation problem example'!$F$32</definedName>
     <definedName name="solver_adj" localSheetId="1" hidden="1">'Optimisation problem example'!$B$18:$B$19</definedName>
     <definedName name="solver_cvg" localSheetId="1" hidden="1">0.0001</definedName>
     <definedName name="solver_drv" localSheetId="1" hidden="1">2</definedName>
@@ -285,7 +276,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
+  </numFmts>
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -316,6 +310,13 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -334,18 +335,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -758,7 +761,7 @@
         <c:title>
           <c:tx>
             <c:rich>
-              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
@@ -790,7 +793,7 @@
             <a:effectLst/>
           </c:spPr>
           <c:txPr>
-            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" wrap="square" anchor="ctr" anchorCtr="1"/>
             <a:lstStyle/>
             <a:p>
               <a:pPr>
@@ -1904,11 +1907,11 @@
       <c r="F4">
         <v>0.36</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="5">
         <f>(D4/C4+E4)</f>
         <v>12.25</v>
       </c>
-      <c r="H4">
+      <c r="H4" s="5">
         <f>G4+$B$13*F4/C4</f>
         <v>147.25</v>
       </c>
@@ -1932,12 +1935,12 @@
       <c r="F5">
         <v>0.36</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="5">
         <f t="shared" ref="G5:G7" si="0">(D5/C5+E5)</f>
         <v>25.444444444444443</v>
       </c>
-      <c r="H5">
-        <f t="shared" ref="H5:H7" si="1">G5+$B$13*F5/C5</f>
+      <c r="H5" s="5">
+        <f t="shared" ref="H5:H6" si="1">G5+$B$13*F5/C5</f>
         <v>145.44444444444446</v>
       </c>
     </row>
@@ -1960,11 +1963,11 @@
       <c r="F6">
         <v>0.2</v>
       </c>
-      <c r="G6">
+      <c r="G6" s="5">
         <f t="shared" si="0"/>
         <v>87.706896551724142</v>
       </c>
-      <c r="H6">
+      <c r="H6" s="5">
         <f t="shared" si="1"/>
         <v>139.43103448275863</v>
       </c>
@@ -1988,11 +1991,11 @@
       <c r="F7" t="s">
         <v>16</v>
       </c>
-      <c r="G7">
+      <c r="G7" s="5">
         <f t="shared" si="0"/>
         <v>11.999999999999998</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="5">
         <f>G7</f>
         <v>11.999999999999998</v>
       </c>
@@ -2028,7 +2031,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A13" s="4" t="s">
+      <c r="A13" t="s">
         <v>24</v>
       </c>
       <c r="B13">
@@ -2037,9 +2040,6 @@
       <c r="C13" t="s">
         <v>25</v>
       </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.45">
-      <c r="A14" s="4"/>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A15" s="3" t="s">
@@ -2264,7 +2264,7 @@
       <c r="B24" t="s">
         <v>52</v>
       </c>
-      <c r="C24" s="5"/>
+      <c r="C24" s="4"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" t="s">

</xml_diff>